<commit_message>
Multiple layers on map, and preliminary interactivity between map markers and basic plots.
</commit_message>
<xml_diff>
--- a/patchr/resources/watchdb.all_tables.xlsx
+++ b/patchr/resources/watchdb.all_tables.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10212"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10312"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tpd0001/github/watch-wv/dap/resources/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tpd0001/github/watch-wv/patchr/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9016CE19-F705-4247-B499-E5C3D1E752A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A118B9A-00E5-354C-BF81-B1C6E72382E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="45940" yWindow="0" windowWidth="31260" windowHeight="27040" activeTab="1" xr2:uid="{ABEE2980-A2EF-284E-9534-8BF6C1D1D8CC}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{ABEE2980-A2EF-284E-9534-8BF6C1D1D8CC}"/>
   </bookViews>
   <sheets>
     <sheet name="location" sheetId="1" r:id="rId1"/>
@@ -1304,7 +1304,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1376,6 +1376,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2684,7 +2687,7 @@
         <v>361</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>103</v>
+        <v>60</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>65</v>
@@ -2899,7 +2902,7 @@
         <v>361</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>103</v>
+        <v>60</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>118</v>
@@ -3329,7 +3332,7 @@
         <v>361</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>103</v>
+        <v>60</v>
       </c>
       <c r="D31" s="2" t="s">
         <v>79</v>
@@ -4403,8 +4406,8 @@
       <c r="B52" s="2" t="s">
         <v>362</v>
       </c>
-      <c r="C52" s="4" t="s">
-        <v>103</v>
+      <c r="C52" s="33" t="s">
+        <v>60</v>
       </c>
       <c r="D52" s="2" t="s">
         <v>189</v>
@@ -4432,8 +4435,8 @@
       <c r="B53" s="2" t="s">
         <v>362</v>
       </c>
-      <c r="C53" s="4" t="s">
-        <v>103</v>
+      <c r="C53" s="33" t="s">
+        <v>60</v>
       </c>
       <c r="D53" s="2" t="s">
         <v>185</v>
@@ -4461,8 +4464,8 @@
       <c r="B54" s="2" t="s">
         <v>362</v>
       </c>
-      <c r="C54" s="4" t="s">
-        <v>103</v>
+      <c r="C54" s="33" t="s">
+        <v>60</v>
       </c>
       <c r="D54" s="2" t="s">
         <v>187</v>
@@ -4490,8 +4493,8 @@
       <c r="B55" s="2" t="s">
         <v>362</v>
       </c>
-      <c r="C55" s="4" t="s">
-        <v>103</v>
+      <c r="C55" s="33" t="s">
+        <v>60</v>
       </c>
       <c r="D55" s="2" t="s">
         <v>68</v>
@@ -4539,8 +4542,8 @@
       <c r="B56" s="2" t="s">
         <v>362</v>
       </c>
-      <c r="C56" s="4" t="s">
-        <v>103</v>
+      <c r="C56" s="33" t="s">
+        <v>60</v>
       </c>
       <c r="D56" s="2" t="s">
         <v>164</v>
@@ -4593,8 +4596,8 @@
       <c r="B57" s="2" t="s">
         <v>362</v>
       </c>
-      <c r="C57" s="4" t="s">
-        <v>103</v>
+      <c r="C57" s="33" t="s">
+        <v>60</v>
       </c>
       <c r="D57" s="2" t="s">
         <v>160</v>
@@ -4647,8 +4650,8 @@
       <c r="B58" s="2" t="s">
         <v>362</v>
       </c>
-      <c r="C58" s="4" t="s">
-        <v>103</v>
+      <c r="C58" s="33" t="s">
+        <v>60</v>
       </c>
       <c r="D58" s="2" t="s">
         <v>155</v>
@@ -4757,8 +4760,8 @@
       <c r="B60" s="2" t="s">
         <v>362</v>
       </c>
-      <c r="C60" s="4" t="s">
-        <v>103</v>
+      <c r="C60" s="33" t="s">
+        <v>60</v>
       </c>
       <c r="D60" s="2" t="s">
         <v>170</v>
@@ -4813,8 +4816,8 @@
       <c r="B61" s="2" t="s">
         <v>362</v>
       </c>
-      <c r="C61" s="4" t="s">
-        <v>103</v>
+      <c r="C61" s="33" t="s">
+        <v>60</v>
       </c>
       <c r="D61" s="2" t="s">
         <v>163</v>
@@ -4867,8 +4870,8 @@
       <c r="B62" s="2" t="s">
         <v>362</v>
       </c>
-      <c r="C62" s="4" t="s">
-        <v>103</v>
+      <c r="C62" s="33" t="s">
+        <v>60</v>
       </c>
       <c r="D62" s="2" t="s">
         <v>179</v>
@@ -4923,8 +4926,8 @@
       <c r="B63" s="2" t="s">
         <v>362</v>
       </c>
-      <c r="C63" s="4" t="s">
-        <v>103</v>
+      <c r="C63" s="33" t="s">
+        <v>60</v>
       </c>
       <c r="D63" s="2" t="s">
         <v>177</v>
@@ -4979,8 +4982,8 @@
       <c r="B64" s="2" t="s">
         <v>362</v>
       </c>
-      <c r="C64" s="4" t="s">
-        <v>103</v>
+      <c r="C64" s="33" t="s">
+        <v>60</v>
       </c>
       <c r="D64" s="2" t="s">
         <v>156</v>

</xml_diff>

<commit_message>
Add site to table.
</commit_message>
<xml_diff>
--- a/patchr/resources/watchdb.all_tables.xlsx
+++ b/patchr/resources/watchdb.all_tables.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tpd0001/github/watch-wv/patchr/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16A27116-A4F4-834A-AB6D-F1644DB3B323}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13269A63-E9F3-264F-8CF3-597B4A05EFE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="51200" yWindow="4760" windowWidth="30240" windowHeight="18980" activeTab="1" xr2:uid="{ABEE2980-A2EF-284E-9534-8BF6C1D1D8CC}"/>
+    <workbookView xWindow="11260" yWindow="1600" windowWidth="30240" windowHeight="18980" xr2:uid="{ABEE2980-A2EF-284E-9534-8BF6C1D1D8CC}"/>
   </bookViews>
   <sheets>
     <sheet name="location" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1622" uniqueCount="653">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1639" uniqueCount="660">
   <si>
     <t>CharlestonWWTP-01</t>
   </si>
@@ -2002,6 +2002,27 @@
   </si>
   <si>
     <t>54067-002-01-00-00</t>
+  </si>
+  <si>
+    <t>CHP</t>
+  </si>
+  <si>
+    <t>Chapmanville</t>
+  </si>
+  <si>
+    <t>ChapmanvilleWWTP</t>
+  </si>
+  <si>
+    <t>Constructed 1970s, small contrubution amount from funeral home. Average sewage travel time "2 hours or a bit more". Not CSO. Sampled 7AM to 3PM after rag and grit removal.</t>
+  </si>
+  <si>
+    <t>Chapmanville WWTP</t>
+  </si>
+  <si>
+    <t>WV0024678</t>
+  </si>
+  <si>
+    <t>54045-001-01-00-00</t>
   </si>
 </sst>
 </file>
@@ -2259,7 +2280,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -2421,6 +2442,13 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -2741,7 +2769,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0856F7A-D0C0-3942-9027-9FB2F3C2C3E0}">
-  <dimension ref="A1:T86"/>
+  <dimension ref="A1:T87"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="31.33203125" customWidth="1"/>
@@ -7693,6 +7721,66 @@
         <v>25703</v>
       </c>
     </row>
+    <row r="87" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A87" s="71" t="s">
+        <v>653</v>
+      </c>
+      <c r="B87" s="71"/>
+      <c r="C87" s="71" t="s">
+        <v>352</v>
+      </c>
+      <c r="D87" s="72" t="s">
+        <v>103</v>
+      </c>
+      <c r="E87" s="71" t="s">
+        <v>654</v>
+      </c>
+      <c r="F87" s="71" t="s">
+        <v>340</v>
+      </c>
+      <c r="G87" s="71" t="s">
+        <v>368</v>
+      </c>
+      <c r="H87" s="71">
+        <v>-82.025433489999998</v>
+      </c>
+      <c r="I87" s="71">
+        <v>37.978467389999999</v>
+      </c>
+      <c r="J87" s="71" t="s">
+        <v>655</v>
+      </c>
+      <c r="K87" s="71" t="s">
+        <v>205</v>
+      </c>
+      <c r="L87" s="73">
+        <v>1200</v>
+      </c>
+      <c r="M87" s="73" t="s">
+        <v>338</v>
+      </c>
+      <c r="N87" s="73">
+        <v>8</v>
+      </c>
+      <c r="O87" s="73">
+        <v>200</v>
+      </c>
+      <c r="P87" s="73">
+        <v>60</v>
+      </c>
+      <c r="Q87" s="71" t="s">
+        <v>347</v>
+      </c>
+      <c r="R87" s="71" t="s">
+        <v>20</v>
+      </c>
+      <c r="S87" s="72">
+        <v>25508</v>
+      </c>
+      <c r="T87" s="71" t="s">
+        <v>656</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:T85" xr:uid="{D0856F7A-D0C0-3942-9027-9FB2F3C2C3E0}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:T86">
@@ -7707,7 +7795,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7706D3C3-8C4A-6E4A-999A-41BCCB2FAC67}">
-  <dimension ref="A1:Z50"/>
+  <dimension ref="A1:Z51"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="27.83203125" bestFit="1" customWidth="1"/>
@@ -9073,6 +9161,32 @@
       </c>
       <c r="I50" s="69">
         <v>4200</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A51" s="15" t="s">
+        <v>655</v>
+      </c>
+      <c r="B51" t="s">
+        <v>659</v>
+      </c>
+      <c r="C51" s="15" t="s">
+        <v>657</v>
+      </c>
+      <c r="E51" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="F51" s="15" t="s">
+        <v>658</v>
+      </c>
+      <c r="G51" s="28">
+        <v>54002315001</v>
+      </c>
+      <c r="H51" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="I51" s="7">
+        <v>1200</v>
       </c>
     </row>
   </sheetData>

</xml_diff>